<commit_message>
feat: editable meal catalog with add/delete via UI
</commit_message>
<xml_diff>
--- a/data/meals.xlsx
+++ b/data/meals.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meals" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="meals" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -419,77 +415,69 @@
   </sheetPr>
   <dimension ref="A1:J25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="75" customWidth="1" min="9" max="9"/>
-    <col width="75" customWidth="1" min="10" max="10"/>
-  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>week</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>meal</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>meal_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>gender</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>kcal</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>protein_g</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>carbs_g</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>fat_g</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>ingredients</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>method</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" t="n">
-        <v>1</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -501,17 +489,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E2" t="n">
-        <v>432</v>
-      </c>
-      <c r="F2" t="n">
-        <v>45.3</v>
-      </c>
-      <c r="G2" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H2" t="n">
-        <v>6</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>432</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>45.3</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -525,11 +521,15 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" t="n">
-        <v>1</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -541,17 +541,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E3" t="n">
-        <v>360</v>
-      </c>
-      <c r="F3" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="G3" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>4.5</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>31.5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -565,11 +573,15 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -581,17 +593,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E4" t="n">
-        <v>395</v>
-      </c>
-      <c r="F4" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="G4" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="H4" t="n">
-        <v>4.8</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>395</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>43.8</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>30.1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -605,11 +625,15 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" t="n">
-        <v>2</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -621,17 +645,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E5" t="n">
-        <v>323</v>
-      </c>
-      <c r="F5" t="n">
-        <v>30</v>
-      </c>
-      <c r="G5" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>3.3</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>30.1</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -645,11 +677,15 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -661,17 +697,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E6" t="n">
-        <v>242</v>
-      </c>
-      <c r="F6" t="n">
-        <v>29.3</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>3</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>29.3</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -685,11 +729,15 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" t="n">
-        <v>3</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -701,17 +749,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E7" t="n">
-        <v>144</v>
-      </c>
-      <c r="F7" t="n">
-        <v>18.7</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>1.7</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>144</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>18.7</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>1.7</t>
+        </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
@@ -725,11 +781,15 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" t="n">
-        <v>1</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -741,17 +801,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E8" t="n">
-        <v>432</v>
-      </c>
-      <c r="F8" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="G8" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H8" t="n">
-        <v>7.7</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>432</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>43.5</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>7.7</t>
+        </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
@@ -765,11 +833,15 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" t="n">
-        <v>1</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -781,17 +853,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E9" t="n">
-        <v>360</v>
-      </c>
-      <c r="F9" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H9" t="n">
-        <v>5.6</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>360</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>30.3</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
@@ -805,11 +885,15 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" t="n">
-        <v>2</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -821,17 +905,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E10" t="n">
-        <v>438</v>
-      </c>
-      <c r="F10" t="n">
-        <v>44.6</v>
-      </c>
-      <c r="G10" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="H10" t="n">
-        <v>4.9</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>438</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>44.6</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>40.2</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
@@ -845,11 +937,15 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" t="n">
-        <v>2</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -861,17 +957,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E11" t="n">
-        <v>366</v>
-      </c>
-      <c r="F11" t="n">
-        <v>30.8</v>
-      </c>
-      <c r="G11" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="H11" t="n">
-        <v>3.3</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>30.8</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>40.2</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -885,11 +989,15 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" t="n">
-        <v>3</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -901,17 +1009,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E12" t="n">
-        <v>302</v>
-      </c>
-      <c r="F12" t="n">
-        <v>39.3</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>5.7</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>302</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>39.3</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -925,11 +1041,15 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B13" t="n">
-        <v>3</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -941,17 +1061,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E13" t="n">
-        <v>242</v>
-      </c>
-      <c r="F13" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>3.9</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>242</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>28.3</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -965,11 +1093,15 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
-        <v>3</v>
-      </c>
-      <c r="B14" t="n">
-        <v>1</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -981,17 +1113,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E14" t="n">
-        <v>463</v>
-      </c>
-      <c r="F14" t="n">
-        <v>41.7</v>
-      </c>
-      <c r="G14" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H14" t="n">
-        <v>10.3</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>463</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>41.7</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1005,11 +1145,15 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
-        <v>3</v>
-      </c>
-      <c r="B15" t="n">
-        <v>1</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1021,17 +1165,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E15" t="n">
-        <v>381</v>
-      </c>
-      <c r="F15" t="n">
-        <v>29.1</v>
-      </c>
-      <c r="G15" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="H15" t="n">
-        <v>7.3</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>381</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>29.1</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1045,11 +1197,15 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
-        <v>3</v>
-      </c>
-      <c r="B16" t="n">
-        <v>2</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1061,17 +1217,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E16" t="n">
-        <v>395</v>
-      </c>
-      <c r="F16" t="n">
-        <v>43.8</v>
-      </c>
-      <c r="G16" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="H16" t="n">
-        <v>4.8</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>395</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>43.8</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>30.1</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1085,11 +1249,15 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
-        <v>3</v>
-      </c>
-      <c r="B17" t="n">
-        <v>2</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1101,17 +1269,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E17" t="n">
-        <v>323</v>
-      </c>
-      <c r="F17" t="n">
-        <v>30</v>
-      </c>
-      <c r="G17" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="H17" t="n">
-        <v>3.3</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>323</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>30.0</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>30.1</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3.3</t>
+        </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1125,11 +1301,15 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
-        <v>3</v>
-      </c>
-      <c r="B18" t="n">
-        <v>3</v>
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1141,17 +1321,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E18" t="n">
-        <v>230</v>
-      </c>
-      <c r="F18" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="G18" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" t="n">
-        <v>3.9</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1165,11 +1353,15 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
-        <v>3</v>
-      </c>
-      <c r="B19" t="n">
-        <v>3</v>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1181,17 +1373,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E19" t="n">
-        <v>170</v>
-      </c>
-      <c r="F19" t="n">
-        <v>23</v>
-      </c>
-      <c r="G19" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" t="n">
-        <v>2.6</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>23.0</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1205,11 +1405,15 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
-        <v>4</v>
-      </c>
-      <c r="B20" t="n">
-        <v>1</v>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1221,17 +1425,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E20" t="n">
-        <v>578</v>
-      </c>
-      <c r="F20" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="G20" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="H20" t="n">
-        <v>7.3</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>578</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>55.1</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>57.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>7.3</t>
+        </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1245,11 +1457,15 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
-        <v>4</v>
-      </c>
-      <c r="B21" t="n">
-        <v>1</v>
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1261,17 +1477,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E21" t="n">
-        <v>506</v>
-      </c>
-      <c r="F21" t="n">
-        <v>41.3</v>
-      </c>
-      <c r="G21" t="n">
-        <v>57.5</v>
-      </c>
-      <c r="H21" t="n">
-        <v>5.8</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>506</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>41.3</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>57.5</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
@@ -1285,11 +1509,15 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
-        <v>4</v>
-      </c>
-      <c r="B22" t="n">
-        <v>2</v>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1301,17 +1529,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E22" t="n">
-        <v>438</v>
-      </c>
-      <c r="F22" t="n">
-        <v>42.8</v>
-      </c>
-      <c r="G22" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="H22" t="n">
-        <v>6.5</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>438</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>42.8</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>40.2</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>6.5</t>
+        </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -1325,11 +1561,15 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
-        <v>4</v>
-      </c>
-      <c r="B23" t="n">
-        <v>2</v>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1341,17 +1581,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E23" t="n">
-        <v>366</v>
-      </c>
-      <c r="F23" t="n">
-        <v>29.6</v>
-      </c>
-      <c r="G23" t="n">
-        <v>40.2</v>
-      </c>
-      <c r="H23" t="n">
-        <v>4.4</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>366</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>29.6</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>40.2</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1365,11 +1613,15 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
-        <v>4</v>
-      </c>
-      <c r="B24" t="n">
-        <v>3</v>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1381,17 +1633,25 @@
           <t>male</t>
         </is>
       </c>
-      <c r="E24" t="n">
-        <v>230</v>
-      </c>
-      <c r="F24" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="G24" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" t="n">
-        <v>3.9</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>230</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>34.5</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>3.9</t>
+        </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1405,11 +1665,15 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
-        <v>4</v>
-      </c>
-      <c r="B25" t="n">
-        <v>3</v>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1421,17 +1685,25 @@
           <t>female</t>
         </is>
       </c>
-      <c r="E25" t="n">
-        <v>170</v>
-      </c>
-      <c r="F25" t="n">
-        <v>23</v>
-      </c>
-      <c r="G25" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" t="n">
-        <v>2.6</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>170</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>23.0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2.6</t>
+        </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>

</xml_diff>